<commit_message>
Eliminated comprobations + changed colors
</commit_message>
<xml_diff>
--- a/Practica_1_StarWars/DataSet.xlsx
+++ b/Practica_1_StarWars/DataSet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\armii\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\armii\Documents\Universidad\Geometria_Computacional\Practicas_GC\Practica_1_StarWars\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20B3479-987C-4F9A-8800-77FFC74C9BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28F33EA-7B50-41C2-8B58-7969401344B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9804" yWindow="0" windowWidth="13332" windowHeight="12336" xr2:uid="{B231091D-8353-4934-ADE5-A67AA9A28C5F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B231091D-8353-4934-ADE5-A67AA9A28C5F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -35,14 +35,18 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -70,8 +74,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27971293-3F87-433E-8B21-3683EF08D433}">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -489,27 +494,21 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
+        <v>-1</v>
+      </c>
+      <c r="B4">
+        <v>13</v>
+      </c>
+      <c r="C4">
         <v>-1.5</v>
       </c>
-      <c r="B4">
+      <c r="D4">
         <v>4</v>
       </c>
-      <c r="C4">
-        <v>-1</v>
-      </c>
-      <c r="D4">
-        <v>13</v>
-      </c>
       <c r="E4">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F4">
-        <v>13</v>
-      </c>
-      <c r="G4">
-        <v>1.5</v>
-      </c>
-      <c r="H4">
         <v>4</v>
       </c>
     </row>
@@ -619,22 +618,22 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>-11.79</v>
+        <v>-11.8</v>
       </c>
       <c r="B9">
-        <v>12.5</v>
+        <v>11.4</v>
       </c>
       <c r="C9">
-        <v>-11.21</v>
+        <v>-11.2</v>
       </c>
       <c r="D9">
-        <v>12.5</v>
+        <v>10</v>
       </c>
       <c r="E9">
         <v>-11.2</v>
       </c>
       <c r="F9">
-        <v>10</v>
+        <v>11.4</v>
       </c>
       <c r="G9">
         <v>-11.8</v>
@@ -1151,7 +1150,7 @@
         <v>-1.8</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>6</v>
       </c>
@@ -1171,7 +1170,7 @@
         <v>-1.8</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>12</v>
       </c>
@@ -1191,7 +1190,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>12</v>
       </c>
@@ -1217,7 +1216,7 @@
         <v>-2.6</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>12.2</v>
       </c>
@@ -1243,7 +1242,7 @@
         <v>-2.6</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>12</v>
       </c>
@@ -1269,7 +1268,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>12</v>
       </c>
@@ -1295,12 +1294,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>11.8</v>
       </c>
       <c r="B39">
-        <v>10</v>
+        <v>11.4</v>
       </c>
       <c r="C39">
         <v>11.2</v>
@@ -1309,17 +1308,38 @@
         <v>10</v>
       </c>
       <c r="E39">
-        <v>11.79</v>
+        <v>11.2</v>
       </c>
       <c r="F39">
-        <v>12.5</v>
+        <v>11.4</v>
       </c>
       <c r="G39">
-        <v>11.21</v>
+        <v>11.8</v>
       </c>
       <c r="H39">
-        <v>12.5</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>-1</v>
+      </c>
+      <c r="B40">
+        <v>13</v>
+      </c>
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40">
+        <v>13</v>
+      </c>
+      <c r="E40">
+        <v>1.5</v>
+      </c>
+      <c r="F40">
+        <v>4</v>
+      </c>
+      <c r="J40" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>